<commit_message>
GridIntensity: add Table 10's GCP-excluded and single-provider rows; GCP PUE cited to the 2026 report [36]
Table 10 now exports in full from the workbook (359 / 47; 319 / 0; all-Azure 73;
gas-only 500 / 500). New typed shares and the 500 gCO2e/kWh scenario intensity are
declared inputs. Audit: 3,954 formulas, 475 declared inputs, 0 undeclared constants.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/workbooks/PUE_Calculation_Aug2026.xlsx
+++ b/data/workbooks/PUE_Calculation_Aug2026.xlsx
@@ -76,7 +76,7 @@
     <t xml:space="preserve">Google Cloud Platform</t>
   </si>
   <si>
-    <t xml:space="preserve">Appendix A.2 [17]: fleet-wide 2024</t>
+    <t xml:space="preserve">Appendix A.2 [36]: fleet-wide 2025 (1.09 in 2024)</t>
   </si>
   <si>
     <t xml:space="preserve">Routing share total</t>
@@ -199,11 +199,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -415,96 +415,96 @@
   <dimension ref="A1:I1000"/>
   <sheetFormatPr defaultColWidth="14.43359375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="80"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="10" style="0" width="8.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="80"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="10" style="1" width="8.71"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="2"/>
+      <c r="I5" s="3"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>11</v>
       </c>
@@ -536,7 +536,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>13</v>
       </c>
@@ -568,7 +568,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
         <v>15</v>
       </c>
@@ -600,7 +600,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
         <v>17</v>
       </c>
@@ -632,152 +632,152 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="4" t="n">
         <f aca="false">SUM(B6:B9)</f>
         <v>0.999</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
       <c r="D11" s="6" t="n">
         <f aca="false">SUM(D6:D9)</f>
         <v>1.11624</v>
       </c>
-      <c r="E11" s="2"/>
+      <c r="E11" s="3"/>
       <c r="F11" s="6" t="n">
         <f aca="false">SUM(F6:F9)</f>
         <v>1.17519</v>
       </c>
-      <c r="G11" s="2"/>
+      <c r="G11" s="3"/>
       <c r="H11" s="6" t="n">
         <f aca="false">SUM(H6:H9)</f>
         <v>1.21449</v>
       </c>
-      <c r="I11" s="2"/>
+      <c r="I11" s="3"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>1.12</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
       <c r="D13" s="5" t="n">
         <f aca="false">D11/$B$12</f>
         <v>0.996642857142857</v>
       </c>
-      <c r="E13" s="2"/>
+      <c r="E13" s="3"/>
       <c r="F13" s="5" t="n">
         <f aca="false">F11/$B$12</f>
         <v>1.04927678571429</v>
       </c>
-      <c r="G13" s="2"/>
+      <c r="G13" s="3"/>
       <c r="H13" s="5" t="n">
         <f aca="false">H11/$B$12</f>
         <v>1.08436607142857</v>
       </c>
-      <c r="I13" s="2"/>
+      <c r="I13" s="3"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
       <c r="D14" s="5" t="n">
         <f aca="false">D13/$F$13</f>
         <v>0.949837898552575</v>
       </c>
-      <c r="E14" s="2"/>
+      <c r="E14" s="3"/>
       <c r="F14" s="5" t="n">
         <f aca="false">F13/$F$13</f>
         <v>1</v>
       </c>
-      <c r="G14" s="2"/>
+      <c r="G14" s="3"/>
       <c r="H14" s="5" t="n">
         <f aca="false">H13/$F$13</f>
         <v>1.03344140096495</v>
       </c>
-      <c r="I14" s="2"/>
+      <c r="I14" s="3"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>